<commit_message>
fix: adjust import script for TK headers, update dropdown options, and fix Pesantren/Yayasan filter format
</commit_message>
<xml_diff>
--- a/docs/program/RKA MA.xlsx
+++ b/docs/program/RKA MA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Download\Laporan Program Pesantren\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Download\Tugas Akhir\Smart_Santri\smart_santri\docs\program\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159F8FB0-8995-443C-8F1F-3E4226490772}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1D4092A-4A1A-4AF1-8E07-8DE1312CCF07}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B3DDAF4A-F012-49A4-9619-7A6A1ACE13E4}"/>
   </bookViews>
@@ -2735,12 +2735,6 @@
     <t>ISI</t>
   </si>
   <si>
-    <t>PROSES</t>
-  </si>
-  <si>
-    <t>PENILAIAN</t>
-  </si>
-  <si>
     <t>KOMPETENSI LULUSAN</t>
   </si>
   <si>
@@ -2753,7 +2747,13 @@
     <t>PENGEMBANGAN PEMBIAYAAN</t>
   </si>
   <si>
-    <t>SARANA DAN PRASARANA</t>
+    <t>PENGEMBANGAN SARANA DAN PRASARANA</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN PROSES</t>
+  </si>
+  <si>
+    <t>PENGEMBANGAN PENILAIAN</t>
   </si>
 </sst>
 </file>
@@ -3408,7 +3408,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>46</v>
@@ -4417,7 +4417,7 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>200</v>
@@ -4636,7 +4636,7 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>229</v>
@@ -5249,7 +5249,7 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="8" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="B106" s="7" t="s">
         <v>318</v>
@@ -5639,7 +5639,7 @@
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="B126" s="6" t="s">
         <v>364</v>
@@ -6973,7 +6973,7 @@
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B194" s="6" t="s">
         <v>543</v>
@@ -7630,7 +7630,7 @@
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" s="8" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="B227" s="7" t="s">
         <v>625</v>

</xml_diff>